<commit_message>
Addressed Carlos comments on jun 3 2026
</commit_message>
<xml_diff>
--- a/Rubrica_Tab1_Detallada_Full_v3.xlsx
+++ b/Rubrica_Tab1_Detallada_Full_v3.xlsx
@@ -855,17 +855,17 @@
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O3" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P3" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
@@ -959,17 +959,17 @@
       </c>
       <c r="N4" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O4" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P4" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q4" s="19" t="inlineStr">
@@ -1065,17 +1065,17 @@
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P5" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -1164,17 +1164,17 @@
       <c r="M6" s="2" t="n"/>
       <c r="N6" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O6" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P6" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
@@ -1268,17 +1268,17 @@
       <c r="M7" s="2" t="n"/>
       <c r="N7" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P7" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q7" s="2" t="n"/>
@@ -1362,17 +1362,17 @@
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O8" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P8" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
@@ -1462,17 +1462,17 @@
       <c r="M9" s="2" t="n"/>
       <c r="N9" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P9" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q9" s="2" t="n"/>
@@ -1557,17 +1557,17 @@
       <c r="M10" s="2" t="n"/>
       <c r="N10" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O10" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P10" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q10" s="2" t="n"/>
@@ -1654,17 +1654,17 @@
       <c r="M11" s="2" t="n"/>
       <c r="N11" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O11" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P11" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
@@ -1763,17 +1763,17 @@
       <c r="M12" s="2" t="n"/>
       <c r="N12" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O12" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P12" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q12" s="2" t="n"/>
@@ -1865,17 +1865,17 @@
       </c>
       <c r="N13" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P13" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
@@ -1964,17 +1964,17 @@
       <c r="M14" s="2" t="n"/>
       <c r="N14" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O14" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P14" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q14" s="2" t="n"/>
@@ -2057,17 +2057,17 @@
       <c r="M15" s="2" t="n"/>
       <c r="N15" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P15" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q15" s="2" t="n"/>
@@ -2157,17 +2157,17 @@
       <c r="M16" s="2" t="n"/>
       <c r="N16" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O16" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P16" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
@@ -2270,22 +2270,23 @@
       </c>
       <c r="N17" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el PRODOC incluye una actividad dedicada a accesibilidad, un indicador de personas con discapacidad atendidas, meta cuantificada y partida presupuestaria para ajustes razonables o lengua de señas.</t>
         </is>
       </c>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el PRODOC identifica necesidades de personas con discapacidad y prevé adaptar materiales, pero no incluye indicador específico, meta o presupuesto dedicado.</t>
         </is>
       </c>
       <c r="P17" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el PRODOC solo menciona a personas con discapacidad en una lista amplia de grupos vulnerables, sin actividad, indicador, meta ni recursos dedicados.</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>Guía: «Guía práctica» n.º 18 — Inclusión de personas con discapacidad.</t>
+          <t>Guía: «Guía práctica» n.º 18 — Inclusión de personas con discapacidad.
+Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
         </is>
       </c>
       <c r="R17" s="20" t="inlineStr">
@@ -2378,17 +2379,17 @@
       <c r="M18" s="2" t="n"/>
       <c r="N18" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O18" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P18" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
@@ -2481,17 +2482,17 @@
       </c>
       <c r="N19" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P19" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
@@ -2594,17 +2595,17 @@
       </c>
       <c r="N20" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O20" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P20" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q20" s="2" t="n"/>
@@ -2702,17 +2703,17 @@
       </c>
       <c r="N21" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P21" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q21" s="19" t="inlineStr">
@@ -2813,22 +2814,23 @@
       </c>
       <c r="N22" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el PRODOC distingue enfoque sensible/responsivo/transformador, plantea acciones para cambiar normas o relaciones de poder de género, mide cambios en roles/decisión y cita guía técnica aplicable.</t>
         </is>
       </c>
       <c r="O22" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el PRODOC tiene talleres para mujeres y lenguaje sensible al género, pero no explica cómo transforma normas, relaciones de poder o barreras estructurales.</t>
         </is>
       </c>
       <c r="P22" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el PRODOC usa formulaciones genéricas de igualdad de género o participación de mujeres, sin acciones transformadoras ni indicadores de cambio relacional.</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>Guía: «Guía práctica» n.º 15 — Incorporación de la perspectiva de género.</t>
+          <t>Guía: «Guía práctica» n.º 15 — Incorporación de la perspectiva de género.
+Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
         </is>
       </c>
       <c r="R22" s="20" t="inlineStr">
@@ -2919,17 +2921,17 @@
       <c r="M23" s="5" t="n"/>
       <c r="N23" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P23" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q23" s="5" t="inlineStr">
@@ -3020,17 +3022,17 @@
       <c r="M24" s="5" t="n"/>
       <c r="N24" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O24" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P24" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q24" s="5" t="n"/>
@@ -3115,17 +3117,17 @@
       <c r="M25" s="5" t="n"/>
       <c r="N25" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P25" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q25" s="5" t="inlineStr">
@@ -3214,17 +3216,17 @@
       <c r="M26" s="5" t="n"/>
       <c r="N26" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O26" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P26" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q26" s="5" t="n"/>
@@ -3316,17 +3318,17 @@
       <c r="M27" s="5" t="n"/>
       <c r="N27" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P27" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q27" s="19" t="inlineStr">
@@ -3421,17 +3423,17 @@
       <c r="M28" s="5" t="n"/>
       <c r="N28" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O28" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P28" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q28" s="5" t="n"/>
@@ -3516,17 +3518,17 @@
       <c r="M29" s="5" t="n"/>
       <c r="N29" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P29" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q29" s="5" t="n"/>
@@ -3611,17 +3613,17 @@
       <c r="M30" s="5" t="n"/>
       <c r="N30" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O30" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P30" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr">
@@ -3708,17 +3710,17 @@
       <c r="M31" s="5" t="n"/>
       <c r="N31" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P31" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q31" s="19" t="inlineStr">
@@ -3815,17 +3817,17 @@
       <c r="M32" s="5" t="n"/>
       <c r="N32" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O32" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P32" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q32" s="5" t="n"/>
@@ -3922,17 +3924,17 @@
       </c>
       <c r="N33" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P33" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q33" s="5" t="n"/>
@@ -4022,17 +4024,17 @@
       <c r="M34" s="5" t="n"/>
       <c r="N34" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O34" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P34" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q34" s="5" t="n"/>
@@ -4119,17 +4121,17 @@
       <c r="M35" s="5" t="n"/>
       <c r="N35" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P35" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q35" s="19" t="inlineStr">
@@ -4225,20 +4227,24 @@
       <c r="M36" s="8" t="n"/>
       <c r="N36" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): la teoría del cambio conecta productos, resultados e impacto con mecanismos causales, supuestos explícitos y evidencia de intervenciones previas; el énfasis está en cambios logrados, no en actividades ejecutadas.</t>
         </is>
       </c>
       <c r="O36" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): existe una cadena productos-resultados-impacto, pero algunos mecanismos causales o supuestos quedan implícitos y la explicación mezcla resultados con actividades.</t>
         </is>
       </c>
       <c r="P36" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
-        </is>
-      </c>
-      <c r="Q36" s="8" t="n"/>
+          <t>Ejemplo orientativo (sintético): el documento enumera actividades y productos sin explicar cómo generan resultados ni qué supuestos sostienen el cambio esperado.</t>
+        </is>
+      </c>
+      <c r="Q36" s="8" t="inlineStr">
+        <is>
+          <t>Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
+        </is>
+      </c>
       <c r="S36" s="25" t="inlineStr">
         <is>
           <t>«teoría del cambio», «ToC», «mecanismo de cambio», «supuesto crítico», «si X entonces Y»</t>
@@ -4320,20 +4326,24 @@
       <c r="M37" s="8" t="n"/>
       <c r="N37" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): cada producto cubre una condición necesaria del resultado, no hay brechas evidentes en la ruta causal y la contribución esperada al impacto está explicitada.</t>
         </is>
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): los productos son relevantes para el resultado, pero falta al menos un componente crítico o la contribución al impacto se enuncia de forma general.</t>
         </is>
       </c>
       <c r="P37" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
-        </is>
-      </c>
-      <c r="Q37" s="8" t="n"/>
+          <t>Ejemplo orientativo (sintético): los productos son actividades desconectadas o demasiado limitadas para sostener los resultados propuestos.</t>
+        </is>
+      </c>
+      <c r="Q37" s="8" t="inlineStr">
+        <is>
+          <t>Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
+        </is>
+      </c>
       <c r="R37" s="20" t="inlineStr">
         <is>
           <t>• [Si] Sí bajado a 1/3 elementos (cliente reconoció subjetividad).</t>
@@ -4420,17 +4430,17 @@
       <c r="M38" s="8" t="n"/>
       <c r="N38" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O38" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P38" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q38" s="8" t="n"/>
@@ -4515,17 +4525,17 @@
       <c r="M39" s="8" t="n"/>
       <c r="N39" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P39" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q39" s="8" t="inlineStr">
@@ -4614,17 +4624,17 @@
       <c r="M40" s="8" t="n"/>
       <c r="N40" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O40" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P40" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q40" s="8" t="inlineStr">
@@ -4711,17 +4721,17 @@
       <c r="M41" s="8" t="n"/>
       <c r="N41" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P41" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q41" s="8" t="inlineStr">
@@ -4814,17 +4824,17 @@
       <c r="M42" s="8" t="n"/>
       <c r="N42" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O42" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P42" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q42" s="8" t="n"/>
@@ -4907,17 +4917,17 @@
       <c r="M43" s="8" t="n"/>
       <c r="N43" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P43" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q43" s="8" t="n"/>
@@ -5009,20 +5019,24 @@
       </c>
       <c r="N44" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): la igualdad de género aparece en resultados o productos, con indicador y meta específica para medir cambio en acceso, condiciones o capacidad de decisión.</t>
         </is>
       </c>
       <c r="O44" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): hay actividades dedicadas a mujeres o desagregación por sexo, pero los resultados/productos no integran explícitamente igualdad de género.</t>
         </is>
       </c>
       <c r="P44" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
-        </is>
-      </c>
-      <c r="Q44" s="8" t="n"/>
+          <t>Ejemplo orientativo (sintético): género aparece solo en antecedentes o grupos beneficiarios, sin resultado, producto, indicador o meta dedicada.</t>
+        </is>
+      </c>
+      <c r="Q44" s="8" t="inlineStr">
+        <is>
+          <t>Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
+        </is>
+      </c>
       <c r="R44" s="20" t="inlineStr">
         <is>
           <t>• [Si] Sí condicional según si la inclusión es explícita o implícita.</t>
@@ -5116,20 +5130,24 @@
       </c>
       <c r="N45" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): la inclusión de personas con discapacidad figura en resultados o productos, con indicador, meta y medidas operativas de accesibilidad.</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el PRODOC prevé alguna adaptación o consulta, pero la inclusión de discapacidad no queda reflejada en resultados/productos ni metas.</t>
         </is>
       </c>
       <c r="P45" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
-        </is>
-      </c>
-      <c r="Q45" s="8" t="n"/>
+          <t>Ejemplo orientativo (sintético): discapacidad aparece solo como mención de grupo vulnerable, sin resultado, producto, actividad dedicada ni recursos.</t>
+        </is>
+      </c>
+      <c r="Q45" s="8" t="inlineStr">
+        <is>
+          <t>Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
+        </is>
+      </c>
       <c r="R45" s="20" t="inlineStr">
         <is>
           <t>• [Si] Sí condicional según si la inclusión es explícita o implícita.</t>
@@ -5214,17 +5232,17 @@
       <c r="M46" s="8" t="n"/>
       <c r="N46" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O46" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P46" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q46" s="8" t="inlineStr">
@@ -5317,17 +5335,17 @@
       <c r="M47" s="8" t="n"/>
       <c r="N47" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P47" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q47" s="8" t="inlineStr">
@@ -5384,15 +5402,16 @@
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t>Comunidad; Medio ambiente; SST</t>
+          <t>Medio ambiente</t>
         </is>
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>A. Identificación de riesgos comunitarios (no solo del personal del proyecto).
-B. Medidas para riesgos físicos (tráfico, materiales peligrosos, contaminación).
-C. Si hay personal de seguridad: protocolo de uso de la fuerza y prevención de abusos.
-D. Mecanismo de queja comunitario.</t>
+          <t>A. Identificación de riesgos comunitarios (no solo del personal del proyecto; no transversal).
+B. Medidas para riesgos físicos y ambientales (tráfico, materiales peligrosos, contaminación; componente transversal: Medio ambiente).
+C. Si hay personal de seguridad: protocolo de uso de la fuerza y prevención de abusos (condicional; no transversal).
+D. Mecanismo de queja comunitario (no transversal).
+Nota: aplicar DEDICADO vs MARCO solo a la evidencia ambiental. No tratar riesgos comunitarios, SST o seguridad como temas transversales.</t>
         </is>
       </c>
       <c r="J48" s="23" t="inlineStr">
@@ -5422,23 +5441,27 @@
       </c>
       <c r="N48" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O48" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P48" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
-        </is>
-      </c>
-      <c r="Q48" s="8" t="n"/>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
+        </is>
+      </c>
+      <c r="Q48" s="8" t="inlineStr">
+        <is>
+          <t>Ajuste v3: riesgos comunitarios/SST/seguridad no son aspectos transversales; solo la parte ambiental invoca el componente transversal.</t>
+        </is>
+      </c>
       <c r="S48" s="25" t="inlineStr">
         <is>
-          <t>«salud y seguridad de la comunidad», «riesgos comunitarios», «mecanismo de queja comunitario»</t>
+          <t>«salud y seguridad de la comunidad», «riesgos comunitarios», «contaminación», «materiales peligrosos», «mecanismo de queja comunitario»</t>
         </is>
       </c>
       <c r="T48" s="27" t="inlineStr">
@@ -5517,17 +5540,17 @@
       <c r="M49" s="8" t="n"/>
       <c r="N49" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P49" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q49" s="8" t="n"/>
@@ -5619,17 +5642,17 @@
       </c>
       <c r="N50" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O50" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P50" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q50" s="19" t="inlineStr">
@@ -5723,20 +5746,24 @@
       <c r="M51" s="8" t="n"/>
       <c r="N51" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): la matriz identifica riesgos específicos del proyecto, con causas, probabilidad, impacto, responsables y mitigaciones vinculadas a cada riesgo.</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): la matriz incluye riesgos relevantes, pero algunos son genéricos o no tienen causa, nivel o mitigación suficientemente específica.</t>
         </is>
       </c>
       <c r="P51" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
-        </is>
-      </c>
-      <c r="Q51" s="8" t="n"/>
+          <t>Ejemplo orientativo (sintético): el documento solo usa categorías amplias como riesgos políticos/económicos sin relación clara con el diseño del proyecto.</t>
+        </is>
+      </c>
+      <c r="Q51" s="8" t="inlineStr">
+        <is>
+          <t>Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
+        </is>
+      </c>
       <c r="S51" s="25" t="inlineStr">
         <is>
           <t>«probabilidad alta/media/baja», «impacto», «escala 1–5»</t>
@@ -5818,17 +5845,17 @@
       <c r="M52" s="8" t="n"/>
       <c r="N52" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O52" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P52" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q52" s="8" t="n"/>
@@ -5919,17 +5946,17 @@
       </c>
       <c r="N53" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P53" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q53" s="8" t="n"/>
@@ -6022,17 +6049,17 @@
       <c r="M54" s="8" t="n"/>
       <c r="N54" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O54" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P54" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q54" s="8" t="n"/>
@@ -6119,17 +6146,17 @@
       <c r="M55" s="8" t="n"/>
       <c r="N55" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P55" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q55" s="8" t="n"/>
@@ -6220,23 +6247,24 @@
       <c r="M56" s="8" t="n"/>
       <c r="N56" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el marco de S&amp;E incluye indicadores SMART para resultados, líneas de base, metas, hitos, desagregación por sexo/discapacidad y fuentes de verificación.</t>
         </is>
       </c>
       <c r="O56" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): hay indicadores y metas, pero faltan líneas de base, hitos o medición específica de género/discapacidad en parte de los resultados.</t>
         </is>
       </c>
       <c r="P56" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el plan de S&amp;E solo cuenta actividades o productos, sin indicadores SMART de resultados ni desagregaciones relevantes.</t>
         </is>
       </c>
       <c r="Q56" s="19" t="inlineStr">
         <is>
           <t>Este es un criterio compuesto crítico — vale la pena reportar el desglose A–F en el output del LLM.
-▸ Pendiente cliente (G56/J56): cuando el donante impone lineamientos de M&amp;E (p. ej. UE, BM), esos lineamientos prevalecen sobre la rúbrica. Revisar elementos A–F con este criterio adicional.</t>
+▸ Pendiente cliente (G56/J56): cuando el donante impone lineamientos de M&amp;E (p. ej. UE, BM), esos lineamientos prevalecen sobre la rúbrica. Revisar elementos A–F con este criterio adicional.
+Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
         </is>
       </c>
       <c r="R56" s="20" t="inlineStr">
@@ -6323,17 +6351,17 @@
       <c r="M57" s="8" t="n"/>
       <c r="N57" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P57" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q57" s="8" t="inlineStr">
@@ -6433,22 +6461,23 @@
       </c>
       <c r="N58" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): si existe inception, el PRODOC define actividades, productos iniciales, responsables, duración, hitos trimestrales y justificación del plazo según capacidades de socios.</t>
         </is>
       </c>
       <c r="O58" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): se mencionan actividades iniciales o arranque, pero no se precisan resultados del período, hitos o relación con capacidades de socios.</t>
         </is>
       </c>
       <c r="P58" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): hay una fase inicial declarada, pero sin actividades, resultados, responsables ni cronograma verificable.</t>
         </is>
       </c>
       <c r="Q58" s="19" t="inlineStr">
         <is>
-          <t>▸ Cliente (I58) reportó alta complejidad para evaluación automatizada. Marcar como criterio de revisión humana prioritaria — la calificación del modelo debe leerse como hipótesis, no veredicto.</t>
+          <t>▸ Cliente (I58) reportó alta complejidad para evaluación automatizada. Marcar como criterio de revisión humana prioritaria — la calificación del modelo debe leerse como hipótesis que requiere revisión humana, no una determinación final.
+Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
         </is>
       </c>
       <c r="R58" s="20" t="inlineStr">
@@ -6537,17 +6566,17 @@
       <c r="M59" s="8" t="n"/>
       <c r="N59" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P59" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q59" s="8" t="n"/>
@@ -6644,17 +6673,17 @@
       </c>
       <c r="N60" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O60" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P60" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q60" s="8" t="n"/>
@@ -6737,17 +6766,17 @@
       <c r="M61" s="8" t="n"/>
       <c r="N61" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O61" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P61" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q61" s="8" t="n"/>
@@ -6832,20 +6861,24 @@
       <c r="M62" s="8" t="n"/>
       <c r="N62" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el PRODOC compara opciones de implementación, explica costos frente a beneficios esperados y justifica por qué la opción seleccionada maximiza valor o eficiencia.</t>
         </is>
       </c>
       <c r="O62" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el presupuesto parece razonable y hay narrativa de eficiencia, pero no compara alternativas ni explicita tradeoffs costo-beneficio.</t>
         </is>
       </c>
       <c r="P62" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
-        </is>
-      </c>
-      <c r="Q62" s="8" t="n"/>
+          <t>Ejemplo orientativo (sintético): no hay análisis de costo-beneficio, ahorro, eficiencia ni justificación de la relación entre recursos y beneficios esperados.</t>
+        </is>
+      </c>
+      <c r="Q62" s="8" t="inlineStr">
+        <is>
+          <t>Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
+        </is>
+      </c>
       <c r="S62" s="25" t="inlineStr">
         <is>
           <t>«análisis de alternativas», «benchmark», «coste-beneficio»</t>
@@ -6927,17 +6960,17 @@
       <c r="M63" s="11" t="n"/>
       <c r="N63" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O63" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P63" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q63" s="11" t="n"/>
@@ -7022,17 +7055,17 @@
       <c r="M64" s="11" t="n"/>
       <c r="N64" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O64" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P64" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q64" s="11" t="n"/>
@@ -7115,17 +7148,17 @@
       <c r="M65" s="11" t="n"/>
       <c r="N65" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O65" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P65" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q65" s="19" t="inlineStr">
@@ -7221,17 +7254,17 @@
       <c r="M66" s="11" t="n"/>
       <c r="N66" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O66" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P66" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q66" s="19" t="inlineStr">
@@ -7331,17 +7364,17 @@
       </c>
       <c r="N67" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O67" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P67" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q67" s="19" t="inlineStr">
@@ -7435,17 +7468,17 @@
       <c r="M68" s="11" t="n"/>
       <c r="N68" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O68" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P68" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q68" s="11" t="n"/>
@@ -7528,17 +7561,17 @@
       <c r="M69" s="11" t="n"/>
       <c r="N69" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O69" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P69" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q69" s="11" t="inlineStr">
@@ -7625,17 +7658,17 @@
       <c r="M70" s="11" t="n"/>
       <c r="N70" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O70" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P70" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q70" s="11" t="n"/>
@@ -7724,17 +7757,17 @@
       </c>
       <c r="N71" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O71" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P71" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q71" s="11" t="n"/>
@@ -7819,20 +7852,24 @@
       <c r="M72" s="11" t="n"/>
       <c r="N72" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): se documenta experiencia previa de socios ejecutores, personal asignado, sistemas administrativos, roles, recursos y medidas de mitigación de brechas de capacidad.</t>
         </is>
       </c>
       <c r="O72" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): los socios y roles están identificados, pero la evidencia de capacidad operativa o medidas ante brechas es limitada.</t>
         </is>
       </c>
       <c r="P72" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
-        </is>
-      </c>
-      <c r="Q72" s="11" t="n"/>
+          <t>Ejemplo orientativo (sintético): el PRODOC asume que los socios ejecutarán eficazmente sin pruebas de experiencia, recursos, sistemas o responsabilidades claras.</t>
+        </is>
+      </c>
+      <c r="Q72" s="11" t="inlineStr">
+        <is>
+          <t>Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
+        </is>
+      </c>
       <c r="S72" s="25" t="inlineStr">
         <is>
           <t>«track record», «proyectos previos», «capacidad demostrada»</t>
@@ -7916,17 +7953,17 @@
       <c r="M73" s="11" t="n"/>
       <c r="N73" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O73" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P73" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q73" s="11" t="n"/>
@@ -8011,17 +8048,17 @@
       <c r="M74" s="11" t="n"/>
       <c r="N74" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O74" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P74" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q74" s="11" t="n"/>
@@ -8108,17 +8145,17 @@
       <c r="M75" s="11" t="n"/>
       <c r="N75" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O75" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P75" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q75" s="11" t="n"/>
@@ -8207,17 +8244,17 @@
       </c>
       <c r="N76" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O76" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P76" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q76" s="11" t="inlineStr">
@@ -8306,17 +8343,17 @@
       <c r="M77" s="14" t="n"/>
       <c r="N77" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="O77" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="P77" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>(v3) — ejemplos no priorizados en esta ronda; los 12 criterios de subjetividad alta ya tienen ejemplos orientativos</t>
         </is>
       </c>
       <c r="Q77" s="14" t="n"/>
@@ -8401,20 +8438,24 @@
       <c r="M78" s="14" t="n"/>
       <c r="N78" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): la redacción es clara, directa y consistente; cada sección aporta información necesaria y no hay repeticiones, contradicciones ni detalles superfluos.</t>
         </is>
       </c>
       <c r="O78" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
+          <t>Ejemplo orientativo (sintético): el documento es comprensible, pero tiene redundancias, secciones demasiado largas o formulaciones que podrían simplificarse.</t>
         </is>
       </c>
       <c r="P78" s="24" t="inlineStr">
         <is>
-          <t>(v3) — ejemplos no requeridos para criterios de baja/media subjetividad; pendiente bootstrap para alta</t>
-        </is>
-      </c>
-      <c r="Q78" s="14" t="n"/>
+          <t>Ejemplo orientativo (sintético): la redacción contiene contradicciones, párrafos genéricos, detalles innecesarios o ideas centrales difíciles de ubicar.</t>
+        </is>
+      </c>
+      <c r="Q78" s="14" t="inlineStr">
+        <is>
+          <t>Ejemplos v3 añadidos: orientativos y sintéticos; no son citas de un PRODOC real.</t>
+        </is>
+      </c>
       <c r="S78" s="25" t="inlineStr">
         <is>
           <t>resumen ejecutivo, subtítulos, longitud de párrafos, tablas vs prosa</t>

</xml_diff>

<commit_message>
feat: T4 de 1.1.1 precisado + base para traducir la rúbrica al inglés
T4 exigía «verbo de contribución» sin excluir los de alineación. Un PRODOC
de Haití obtuvo Yes con estabilidad 100% enlazando los P&B sólo con
«Aligned with», y los dos «will contribute to» del texto apuntaban a
destinos no citados en T1/T2/T3. Ahora T4 exige que el verbo rija un
destino citado, y excluye explícitamente alineación y coherencia. Las
DECISIONES no cambian: la regla de Parcial (T1∧T2∧T3)∧¬T4 ya cubría el caso.

Traducción: columnas «… (EN)» en el xlsx, sólo para mostrar. La evaluación
usa siempre la columna española (autoritativa), de modo que el idioma no
puede alterar un veredicto. Celda (EN) vacía -> se muestra la española.
Traducidos: los 76 criterios y las 22 preguntas orientadoras distintas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Rubrica_Tab1_Detallada_Full_v3.xlsx
+++ b/Rubrica_Tab1_Detallada_Full_v3.xlsx
@@ -653,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T78"/>
+  <dimension ref="A1:V78"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" style="17" min="1" max="1"/>
@@ -781,6 +781,16 @@
           <t>Subjetividad residual (v3)</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Criterio a evaluar (EN)</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Pregunta orientadora (CONTEXTO — no evaluar) (EN)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="320" customHeight="1" s="17">
       <c r="A3" s="2" t="inlineStr">
@@ -837,7 +847,10 @@
 T1: ¿Cita al menos un resultado/prioridad de P&amp;B con código o nombre? (sí/no)
 T2: ¿Cita al menos un resultado DWCP con nombre del país? (sí/no)
 T3: ¿Cita al menos un CPO por código (formato letra+número, p.ej. ABC-101)? (sí/no)
-T4: ¿El texto vincula la intervención a T1/T2/T3 con verbo de contribución («contribuye», «aporta», «alimenta», «se traduce en»)? (sí/no)
+T4: ¿El texto vincula la intervención a T1/T2/T3 con un verbo de CONTRIBUCIÓN cuyo destino sea uno de los resultados citados en T1, T2 o T3? (sí/no)
+    Cuentan: «contribuye a», «aporta a», «alimenta», «se traduce en», «apoya el logro de» y sus equivalentes en el idioma del documento («contributes to», «feeds into», «translates into», «supports the achievement of»).
+    NO cuentan: verbos de mera alineación o coherencia —«alineado con», «coherente con», «en línea con», «responde a», «aligned with», «consistent with», «in line with»—, porque declaran correspondencia, no aportación.
+    NO cuenta tampoco un verbo de contribución cuyo destino sea un objetivo genérico (p.ej. «contribuirá a resultados más sostenibles en el país») o una entidad no citada en T1/T2/T3: el destino debe ser el resultado P&amp;B, DWCP o CPO identificado.
 DECISIÓN: T1 ∧ T2 ∧ T3 ∧ T4</t>
         </is>
       </c>
@@ -870,7 +883,8 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Verificar también el anexo de marco lógico — los CPO suelen aparecer ahí.</t>
+          <t>Verificar también el anexo de marco lógico — los CPO suelen aparecer ahí.
+27 ago 2026 — T4 precisado: se excluyen los verbos de alineación («alineado con», «aligned with») y se exige que el verbo de contribución rija un destino citado en T1/T2/T3. Motivo: un PRODOC de Haití obtuvo Yes con estabilidad 100% enlazando los P&amp;B sólo con «Aligned with»; la regla de Parcial (T1∧T2∧T3)∧¬T4 ya contemplaba ese caso, pero T4 se leía con demasiada holgura. Las DECISIONES no cambian.</t>
         </is>
       </c>
       <c r="S3" s="25" t="inlineStr">
@@ -881,6 +895,16 @@
       <c r="T3" s="26" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>The intervention specifies its contribution to the ILO's long-term priorities, to P&amp;B outcomes and to DWCP outcomes, including the relevant CPOs.</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Is the overall objective of the programme/project clearly defined?</t>
         </is>
       </c>
     </row>
@@ -993,6 +1017,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>The level of ambition and visibility on disability inclusion is on a par with the disability inclusion marker of the corresponding CPOs.</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Is the overall objective of the programme/project clearly defined?</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="320" customHeight="1" s="17">
       <c r="A5" s="2" t="inlineStr">
@@ -1093,6 +1127,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>The level of ambition and visibility on gender equality is on a par with the gender equality marker of the corresponding CPOs.</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Is the overall objective of the programme/project clearly defined?</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="320" customHeight="1" s="17">
       <c r="A6" s="2" t="inlineStr">
@@ -1197,6 +1241,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>The proposal explains how the project fits within the country's wider development assistance framework, including national development plans.</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Does the project identify the relevant SDGs, UN cooperation frameworks and national frameworks?</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="320" customHeight="1" s="17">
       <c r="A7" s="2" t="inlineStr">
@@ -1292,6 +1346,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>The proposal is consistent with the United Nations Cooperation Framework and contributes to the specific areas for which the ILO is responsible.</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Does the project identify the relevant SDGs, UN cooperation frameworks and national frameworks?</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="320" customHeight="1" s="17">
       <c r="A8" s="2" t="inlineStr">
@@ -1388,6 +1452,16 @@
       <c r="T8" s="26" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>The proposal identifies the relevant SDG indicators, consistent with the SDG indicators linked to the relevant CPOs.</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Does the project identify the relevant SDGs, UN cooperation frameworks and national frameworks?</t>
         </is>
       </c>
     </row>
@@ -1486,6 +1560,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>A problem statement has been formulated on the basis of a situation analysis (baseline study or other evidence).</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Is the proposed intervention relevant to addressing the problem?</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="320" customHeight="1" s="17">
       <c r="A10" s="2" t="inlineStr">
@@ -1579,6 +1663,16 @@
       <c r="T10" s="27" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>The causes of the problem are explained.</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Is the proposed intervention relevant to addressing the problem?</t>
         </is>
       </c>
     </row>
@@ -1689,6 +1783,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>The affected population group / final beneficiaries have been identified, with an analysis of gender roles, division of labour, and the opportunities and constraints facing women and men.</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Is the proposed intervention relevant to addressing the problem?</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="320" customHeight="1" s="17">
       <c r="A12" s="2" t="inlineStr">
@@ -1787,6 +1891,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>The stakeholders related to the problem and the solution have been identified, together with their constraints and interests. The analysis is gender-sensitive and includes, where applicable, women's organizations and organizations of persons with disabilities.</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Is the proposed intervention relevant to addressing the problem?</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="320" customHeight="1" s="17">
       <c r="A13" s="2" t="inlineStr">
@@ -1893,6 +2007,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>The project includes meaningful consultation with all affected stakeholders, especially marginalised and excluded groups. It ensures equitable participation and avoids discriminatory effects on persons with disabilities, indigenous communities, women and other groups.</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Is the proposed intervention relevant to addressing the problem?</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="320" customHeight="1" s="17">
       <c r="A14" s="2" t="inlineStr">
@@ -1988,6 +2112,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>The proposal highlights the ILO's normative and tripartite identity, its capacity and its added value for carrying out the project.</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Does the proposal emphasise the ILO's comparative advantage?</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="320" customHeight="1" s="17">
       <c r="A15" s="2" t="inlineStr">
@@ -2084,6 +2218,16 @@
       <c r="T15" s="26" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>The ILO's presence in the country is highlighted, as well as its portfolio of past and ongoing projects.</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Does the proposal emphasise the ILO's comparative advantage?</t>
         </is>
       </c>
     </row>
@@ -2189,6 +2333,16 @@
       <c r="T16" s="27" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>The proposal presents previous experience and lessons learned from relevant evaluations, and explains how these have shaped the strategy.</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Does the proposal emphasise the ILO's comparative advantage?</t>
         </is>
       </c>
     </row>
@@ -2305,6 +2459,16 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>The project has taken into account the needs and concerns of persons with disabilities.</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Does the proposal reflect the ILO's cross-cutting policy drivers?</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="320" customHeight="1" s="17">
       <c r="A18" s="2" t="inlineStr">
@@ -2407,6 +2571,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>The proposal integrates the relevant ILO Conventions and Recommendations into the project's strategy, indicators and objectives, promoting ratification, application and awareness. References to NORMLEX or other legal sources are included.</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Does the proposal reflect the ILO's cross-cutting policy drivers?</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="320" customHeight="1" s="17">
       <c r="A19" s="2" t="inlineStr">
@@ -2514,6 +2688,16 @@
       <c r="T19" s="27" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Reference is made to the reports of the country-specific supervisory bodies and to the relevant international labour standards in the justification and the implementation strategy.</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Does the proposal reflect the ILO's cross-cutting policy drivers?</t>
         </is>
       </c>
     </row>
@@ -2624,6 +2808,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>The proposal ensures compliance with ILO labour standards (fair wages, safe conditions, fundamental rights). Where workers are engaged directly or through third parties, protective measures and accessible grievance mechanisms apply.</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Does the proposal reflect the ILO's cross-cutting policy drivers?</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="320" customHeight="1" s="17">
       <c r="A21" s="2" t="inlineStr">
@@ -2734,6 +2928,16 @@
       <c r="T21" s="27" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>The proposal gives priority to environmental sustainability, integrating safety and protection measures, assessing impacts on biodiversity and communities, and promoting environmentally sustainable practices.</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Does the proposal reflect the ILO's cross-cutting policy drivers?</t>
         </is>
       </c>
     </row>
@@ -2871,6 +3075,16 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Wherever possible, the proposal promotes and highlights the use of a gender-transformative approach.</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Does the proposal reflect the ILO's cross-cutting policy drivers?</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="320" customHeight="1" s="17">
       <c r="A23" s="5" t="inlineStr">
@@ -2972,6 +3186,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>The proposal describes the process by which constituents and other stakeholders were involved in the design, and refers specifically to their role in monitoring and implementation.</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Have the tripartite partners and other key stakeholders been involved in the design?</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="320" customHeight="1" s="17">
       <c r="A24" s="5" t="inlineStr">
@@ -3069,6 +3293,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Key stakeholders are clearly identified and presented in relation to their link with the final beneficiaries and their role regarding the problem and the proposed solution.</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>Have the tripartite partners and other key stakeholders been involved in the design?</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="320" customHeight="1" s="17">
       <c r="A25" s="5" t="inlineStr">
@@ -3168,6 +3402,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>ACT/EMP and ACTRAV specialists have been consulted.</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>Have the tripartite partners and other key stakeholders been involved in the design?</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="320" customHeight="1" s="17">
       <c r="A26" s="5" t="inlineStr">
@@ -3267,6 +3511,16 @@
       <c r="T26" s="27" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>The proposal describes consultations and agreements with partners and their willingness to contribute to the results (intention to reform, staff time for training, implementation of changes, etc.).</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>Is there ownership of the project by the target groups?</t>
         </is>
       </c>
     </row>
@@ -3374,6 +3628,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Each partner has accepted the project's objectives and targets (as applicable), the performance framework, and the corresponding obligations and responsibilities.</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>Is there ownership of the project by the target groups?</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="320" customHeight="1" s="17">
       <c r="A28" s="5" t="inlineStr">
@@ -3470,6 +3734,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>The proposal explains the strategy by which stakeholder ownership will be fostered and secured on an ongoing basis.</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>Is there ownership of the project by the target groups?</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="320" customHeight="1" s="17">
       <c r="A29" s="5" t="inlineStr">
@@ -3565,6 +3839,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>A capacity assessment of the target groups has been carried out or is planned, and its conclusions are explicitly referred to and integrated into the design.</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>Does the proposal set out a clear and holistic approach to capacity development?</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="320" customHeight="1" s="17">
       <c r="A30" s="5" t="inlineStr">
@@ -3664,6 +3948,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>The proposal sets out its approach to capacity development, addressing individual (technical), organizational and enabling-environment (policy) capacities.</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>Does the proposal set out a clear and holistic approach to capacity development?</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="320" customHeight="1" s="17">
       <c r="A31" s="5" t="inlineStr">
@@ -3764,6 +4058,16 @@
       <c r="T31" s="27" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>It is clear from the proposal that constituents and/or other stakeholders have demonstrated strong interest in contributing to the achievement of results after the project ends.</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>Will the beneficiaries be able to sustain the results?</t>
         </is>
       </c>
     </row>
@@ -3869,6 +4173,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>The proposal includes plans to ensure sustainability of the results after completion (training of trainers, partnerships with local actors, etc.).</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Will the beneficiaries be able to sustain the results?</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="320" customHeight="1" s="17">
       <c r="A33" s="5" t="inlineStr">
@@ -3976,6 +4290,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>In the pilot phase, the proposal identifies the preconditions needed to scale up the approach and sets out the approach for objectively demonstrating its success.</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>Will the beneficiaries be able to sustain the results?</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="320" customHeight="1" s="17">
       <c r="A34" s="5" t="inlineStr">
@@ -4069,6 +4393,16 @@
       <c r="T34" s="27" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>The proposal makes it plausible that the necessary resources (human and financial) will be available once the project has ended.</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>Will the beneficiaries be able to sustain the results?</t>
         </is>
       </c>
     </row>
@@ -4177,6 +4511,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>The project includes an exit strategy setting out plans for the transfer of responsibilities and for capacity development so that national partners can sustain the results.</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>Will the beneficiaries be able to sustain the results?</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="320" customHeight="1" s="17">
       <c r="A36" s="8" t="inlineStr">
@@ -4278,6 +4622,16 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>The causal relationships, mechanisms of change and assumptions between outputs, outcomes and impact are explained clearly and convincingly. The emphasis is on the achievement of results (not on carrying out activities).</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>Is the theory of change clearly expressed?</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="320" customHeight="1" s="17">
       <c r="A37" s="8" t="inlineStr">
@@ -4382,6 +4736,16 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>The outputs appear sufficient for the likely achievement of the outcomes. The expected contribution of the outcomes to impact is also clear.</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>Is the theory of change clearly expressed?</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="320" customHeight="1" s="17">
       <c r="A38" s="8" t="inlineStr">
@@ -4477,6 +4841,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>It is clear from the theory of change which actors will benefit from capacity development and how this is expected to lead to results (improved performance, behavioural change, etc.).</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>Is the theory of change clearly expressed?</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="320" customHeight="1" s="17">
       <c r="A39" s="8" t="inlineStr">
@@ -4576,6 +4950,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Key assumptions are identified, including the results of past, ongoing or planned interventions (including those of other actors).</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>Is the theory of change clearly expressed?</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="320" customHeight="1" s="17">
       <c r="A40" s="8" t="inlineStr">
@@ -4675,6 +5059,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Previous experience gathered from evaluations is cited as evidence to support the intended causal relationship between outputs, outcomes and impact.</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Is the theory of change clearly expressed?</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="320" customHeight="1" s="17">
       <c r="A41" s="8" t="inlineStr">
@@ -4770,6 +5164,16 @@
       <c r="T41" s="26" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>'Change language' is used rather than 'action language' ('through this and that', 'by doing this and that').</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Do the results statements describe concrete situations?</t>
         </is>
       </c>
     </row>
@@ -4871,6 +5275,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>The outcomes (immediate objectives) state the end situation, the conditions of observation and the standard to be met. They are SMART (specific, measurable, achievable, relevant, time-bound).</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>Do the results statements describe concrete situations?</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="320" customHeight="1" s="17">
       <c r="A43" s="8" t="inlineStr">
@@ -4962,6 +5376,16 @@
       <c r="T43" s="26" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>The output statements refer to the result of the activities, not to the activities themselves.</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>Do the results statements describe concrete situations?</t>
         </is>
       </c>
     </row>
@@ -5075,6 +5499,16 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Gender equality is reflected at outcome and/or output level.</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>Have gender equality and disability inclusion been mainstreamed into the logical framework?</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="320" customHeight="1" s="17">
       <c r="A45" s="8" t="inlineStr">
@@ -5186,6 +5620,16 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>The inclusion of persons with disabilities is reflected at outcome and/or output level.</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>Have gender equality and disability inclusion been mainstreamed into the logical framework?</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="320" customHeight="1" s="17">
       <c r="A46" s="8" t="inlineStr">
@@ -5281,6 +5725,16 @@
       <c r="T46" s="26" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>The proposal contains a narrative summary / analysis of the risks.</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>Have the risks been assessed and mitigation measures proposed?</t>
         </is>
       </c>
     </row>
@@ -5386,6 +5840,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>The proposal assesses and mitigates the risks of sexual exploitation and abuse (SEA), including labour influx, power dynamics and exposure to unsafe environments. Prevention mechanisms are in place.</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>Have the risks been assessed and mitigation measures proposed?</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="320" customHeight="1" s="17">
       <c r="A48" s="8" t="inlineStr">
@@ -5492,6 +5956,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>The proposal identifies and mitigates risks to community health and safety (pollution, traffic, hazardous materials). Where security personnel are engaged, measures are in place to prevent abuse.</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>Have the risks been assessed and mitigation measures proposed?</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="320" customHeight="1" s="17">
       <c r="A49" s="8" t="inlineStr">
@@ -5592,6 +6066,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Compliance risks relating to labour standards and to the observations of the supervisory bodies are mentioned/assessed.</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>Have the risks been assessed and mitigation measures proposed?</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="320" customHeight="1" s="17">
       <c r="A50" s="8" t="inlineStr">
@@ -5696,6 +6180,16 @@
       <c r="T50" s="26" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>For projects with a budget above USD 1 million, the latest version of the risk register has been completed and attached to the proposal.</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>Have the risks been assessed and mitigation measures proposed?</t>
         </is>
       </c>
     </row>
@@ -5797,6 +6291,16 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>The risks identified are relevant and sufficiently specific to be meaningful.</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>Have the risks been assessed and mitigation measures proposed?</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="320" customHeight="1" s="17">
       <c r="A52" s="8" t="inlineStr">
@@ -5890,6 +6394,16 @@
       <c r="T52" s="27" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Relevant measures are proposed to address and monitor medium- and high-level risks.</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>Have the risks been assessed and mitigation measures proposed?</t>
         </is>
       </c>
     </row>
@@ -5999,6 +6513,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>The M&amp;E section describes the system planned for collecting information accurately and in good time, justifying the resources. It includes an evaluability review (mandatory for large budgets).</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>Have adequate monitoring and evaluation arrangements been established?</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="320" customHeight="1" s="17">
       <c r="A54" s="8" t="inlineStr">
@@ -6096,6 +6620,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>The feedback loop from progress information into management decisions is described, clearly identifying the information needs for performance reporting. The responsible staff are identified.</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>Have adequate monitoring and evaluation arrangements been established?</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="320" customHeight="1" s="17">
       <c r="A55" s="8" t="inlineStr">
@@ -6191,6 +6725,16 @@
       <c r="T55" s="26" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>The M&amp;E plan has been developed with well-identified information needs. The collection and analysis methods are technically sound. It specifies roles and responsibilities.</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>Have adequate monitoring and evaluation arrangements been established?</t>
         </is>
       </c>
     </row>
@@ -6305,6 +6849,16 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>The M&amp;E plan includes SMART and gender-sensitive indicators, baselines, targets and milestones (which also allow for the inclusion of persons with disabilities and/or other vulnerable groups). The indicators measure the intended results.</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>Have adequate monitoring and evaluation arrangements been established?</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="320" customHeight="1" s="17">
       <c r="A57" s="8" t="inlineStr">
@@ -6407,6 +6961,16 @@
       <c r="T57" s="26" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>The M&amp;E budget complies with ILO guidance. The evaluation budget appears as a separate line and is appropriate to the size/duration (approximately 2% of the total budget).</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>Have adequate monitoring and evaluation arrangements been established?</t>
         </is>
       </c>
     </row>
@@ -6518,6 +7082,16 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>Where there is an inception period, the proposal presents the activities and results of that period. The timeframe is sufficient, considering partners' capacities, complexity and the dynamics of change.</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>Can all results be achieved within the timeframe and budget?</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="320" customHeight="1" s="17">
       <c r="A59" s="8" t="inlineStr">
@@ -6617,6 +7191,16 @@
       <c r="T59" s="27" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>There is clear evidence that the budget is based on an analysis of each activity and includes all the necessary resources.</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>Can all results be achieved within the timeframe and budget?</t>
         </is>
       </c>
     </row>
@@ -6720,6 +7304,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Where applicable, the budget includes provision for specific expertise (gender, disability) and for means that promote inclusion (local languages, sign language, accessibility).</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>Can all results be achieved within the timeframe and budget?</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="320" customHeight="1" s="17">
       <c r="A61" s="8" t="inlineStr">
@@ -6811,6 +7405,16 @@
       <c r="T61" s="26" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>The proposal refers to cost-effectiveness considerations.</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>Is there evidence that cost-effectiveness / value for money has been considered?</t>
         </is>
       </c>
     </row>
@@ -6912,6 +7516,16 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>The proposal shows that the most appropriate balance has been struck between spending/saving costs and increasing/decreasing benefits.</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>Is there evidence that cost-effectiveness / value for money has been considered?</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="320" customHeight="1" s="17">
       <c r="A63" s="11" t="inlineStr">
@@ -7007,6 +7621,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Projects with regional/national results are managed by the field office closest to the beneficiaries. Projects managed centrally from headquarters justify that decision on grounds of effectiveness, cost-effectiveness, capacities, etc.</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>Are the management arrangements clear and adequate?</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="320" customHeight="1" s="17">
       <c r="A64" s="11" t="inlineStr">
@@ -7102,6 +7726,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>The roles and responsibilities of project staff are clearly defined. There is a clear line of accountability and supervision, and the responsible ILO official is identified.</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>Are the management arrangements clear and adequate?</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="320" customHeight="1" s="17">
       <c r="A65" s="11" t="inlineStr">
@@ -7202,6 +7836,16 @@
       <c r="T65" s="27" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Support from headquarters technical or administrative units and/or direct working teams has been budgeted for.</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>Are the management arrangements clear and adequate?</t>
         </is>
       </c>
     </row>
@@ -7310,6 +7954,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>The implementation arrangements (staffing, procurement, financial systems and authorities) are clearly defined.</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>Are the management arrangements clear and adequate?</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="320" customHeight="1" s="17">
       <c r="A67" s="11" t="inlineStr">
@@ -7420,6 +8074,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Where there are contractors, subcontractors or external suppliers, the proposal states that they adhere to decent work and fair employment principles. Grievance mechanisms and compliance monitoring are in place.</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>Are the management arrangements clear and adequate?</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="320" customHeight="1" s="17">
       <c r="A68" s="11" t="inlineStr">
@@ -7515,6 +8179,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>The responsibilities and roles of the participating institutions and partners are clearly defined. Implementation procedures are in place. The proposal states why particular institutions have been selected.</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>Are the implementation arrangements clear?</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="320" customHeight="1" s="17">
       <c r="A69" s="11" t="inlineStr">
@@ -7612,6 +8286,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>The proposal states whether the participating partners have accepted their roles and responsibilities.</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>Are the implementation arrangements clear?</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="320" customHeight="1" s="17">
       <c r="A70" s="11" t="inlineStr">
@@ -7703,6 +8387,16 @@
       <c r="T70" s="26" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>An organizational capacity assessment of the implementing partners has been or will be carried out, and is referred to in the proposal.</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>Are the implementation arrangements clear?</t>
         </is>
       </c>
     </row>
@@ -7804,6 +8498,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>Where necessary, a capacity development plan for the implementing partners is included, including gender responsiveness.</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>Are the implementation arrangements clear?</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="320" customHeight="1" s="17">
       <c r="A72" s="11" t="inlineStr">
@@ -7901,6 +8605,16 @@
       <c r="T72" s="28" t="inlineStr">
         <is>
           <t>Alta</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>The proposal presents sufficient evidence that the implementing partners will ensure effective delivery of the project.</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>Are the implementation arrangements clear?</t>
         </is>
       </c>
     </row>
@@ -8000,6 +8714,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>The project describes how data and results (including evaluation findings) will be communicated to stakeholders, and has allocated adequate resources.</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>Is there a strategy for communicating progress to stakeholders on an ongoing basis?</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="320" customHeight="1" s="17">
       <c r="A74" s="11" t="inlineStr">
@@ -8093,6 +8817,16 @@
       <c r="T74" s="27" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>The proposal has a public communication strategy (general public, human-interest angle) or information on how and when one will be developed.</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>Is there a budgeted communication strategy?</t>
         </is>
       </c>
     </row>
@@ -8192,6 +8926,16 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>Adequate resources (human and financial) are allocated for developing and implementing the strategy. The products are accessible to key stakeholders (alternative formats for persons with disabilities, local languages).</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>Is there a budgeted communication strategy?</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="320" customHeight="1" s="17">
       <c r="A76" s="11" t="inlineStr">
@@ -8295,6 +9039,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>Where the project exceeds USD 5 million and is funded through a PPP or by the European Commission, a communication strategy template has been completed with DCOMM and the country office.</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>Is there a budgeted communication strategy?</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="320" customHeight="1" s="17">
       <c r="A77" s="14" t="inlineStr">
@@ -8390,6 +9144,16 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>All sections have been completed and ordered in line with the guidance materials.</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>Does the proposal follow the template?</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="320" customHeight="1" s="17">
       <c r="A78" s="14" t="inlineStr">
@@ -8487,6 +9251,16 @@
       <c r="T78" s="28" t="inlineStr">
         <is>
           <t>Alta</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>The quality of drafting is high; there is no superfluous detail; the core ideas are written clearly and directly.</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>Is the proposal written clearly and concisely?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rúbrica íntegramente traducida — el xlsx en inglés ya no mezcla idiomas
Traducidas las columnas restantes: Elementos a verificar, Rúbrica —
Parcial / No / No aplica, y Anclas verificables. Barrido automático sobre
una corrida real de 76 criterios: ninguna de las tres hojas conserva texto
español.

Los símbolos lógicos (∧ ∨ ¬ ≥ ≤) coinciden carácter a carácter entre las
columnas española e inglesa en los 76 criterios de Parcial y No: cero
discrepancias. Las anclas se dan con sus equivalentes ingleses, y conservan
códigos, regex, siglas y URLs.

La salida en español sigue siendo idéntica byte a byte a la del baseline.

PENDIENTE: la traducción es mía y necesita revisión de un bilingüe antes de
uso externo. No afecta veredictos —la evaluación lee siempre la columna
española— pero sí a lo que el lector cree que se verificó.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Rubrica_Tab1_Detallada_Full_v3.xlsx
+++ b/Rubrica_Tab1_Detallada_Full_v3.xlsx
@@ -653,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W78"/>
+  <dimension ref="A1:AB78"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" style="17" min="1" max="1"/>
@@ -796,6 +796,31 @@
           <t>Rúbrica — Sí (EN)</t>
         </is>
       </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Elementos a verificar (EN)</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Rúbrica — Parcial (EN)</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Rúbrica — No (EN)</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Rúbrica — No aplica (EN)</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Anclas verificables (v3) (EN)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="320" customHeight="1" s="17">
       <c r="A3" s="2" t="inlineStr">
@@ -925,6 +950,30 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4</t>
         </is>
       </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>A. Explicit citation of P&amp;B priorities / ILO outcomes.
+B. Explicit citation of the country's DWCP outcomes.
+C. Identifies at least one relevant CPO by code or name.
+D. Explains HOW the intervention contributes to A/B/C (not merely a list).</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>DECISION: (T1 ∧ T2 ∧ T3) ∧ ¬T4   (cites everything but does not articulate contribution)
+    OR    (exactly 2 of T1/T2/T3) ∧ T4</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>DECISION: (≤1 of T1/T2/T3 true)   OR   no detectable contribution verb</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>P&amp;B; DWCP; CPO; "contributes to", "aligns with", "feeds into"; CPO codes (e.g. ABC-101)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="320" customHeight="1" s="17">
       <c r="A4" s="2" t="inlineStr">
@@ -1055,6 +1104,33 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>A. Identifies the disability label/marker of the CPOs referenced.
+B. The proposal presents DEDICATED disability actions (not merely a mention).
+C. The level (visibility and ambition) matches the CPO label.</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬T3   (acknowledges the label but the level falls short)</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   OR   ¬T2 (FRAMING only, nothing DEDICATED)</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Only if the CPOs explicitly referenced carry no disability label — this must be documented.</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>"disability label"; "disability marker"; "disability principal/significant/limited"; CPO names with their marker</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="320" customHeight="1" s="17">
       <c r="A5" s="2" t="inlineStr">
@@ -1175,6 +1251,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>A. Identifies the CPO gender marker (0/1/2/3 or equivalent).
+B. The proposal presents DEDICATED gender actions.
+C. The level matches the CPO marker.</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   OR   marker ≥2 ∧ nothing DEDICATED</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>"gender marker"; "GEM"; "principal/significant/limited"; CPO code with marker</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="320" customHeight="1" s="17">
       <c r="A6" s="2" t="inlineStr">
@@ -1298,6 +1396,28 @@
 DECISION: (T1 ∨ T2) ∧ T3</t>
         </is>
       </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>A. Identifies the current national development plan (by name).
+B. Identifies the UN cooperation framework (UNSDCF/equivalent).
+C. Articulates how the project fits within A and B.</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>DECISION: (T1 ∨ T2) ∧ ¬T3   (names a framework but does not articulate the fit)</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ ¬T2   (names no specific framework)</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>"UNSDCF"; "UNDAF"; official name of the national plan; "National Development Plan"; "National Strategy"</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="320" customHeight="1" s="17">
       <c r="A7" s="2" t="inlineStr">
@@ -1412,6 +1532,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>A. Identifies the UNSDCF outcomes/areas to which it contributes.
+B. Identifies the areas where the ILO is the responsible or convening agency.
+C. Articulates the project's contribution to A and B.</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬(T2 ∧ T3)</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   (only generic consistency with the UNSDCF)</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>"UNSDCF Outcome", "UNSDCF Outcome X", "ILO leads", "ILO convenes"</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="320" customHeight="1" s="17">
       <c r="A8" s="2" t="inlineStr">
@@ -1526,6 +1668,28 @@
 T1: Does it cite ≥2 SDG indicators by code (N.N.N format, such as 8.5.2, 1.3.1)? (yes/no)
 T2: Do those indicators appear in the logical framework or the M&amp;E plan? (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>A. Identifies SDG indicators by code (e.g. 8.5.2, 1.3.1).
+B. Those indicators correspond to the SDGs already linked to the CPOs.
+C. The SDG indicators appear in the logical framework or the M&amp;E plan.</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   (cites codes but they are not integrated into M&amp;E)</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   (names only SDGs "5", "8" without indicator codes)</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>regex pattern \d+\.\d+\.\d+ ; "SDG indicator"; "SDG marker"</t>
         </is>
       </c>
     </row>
@@ -1644,6 +1808,28 @@
 DECISION: T1 ∧ T2 ∧ (T3 ∨ T4)</t>
         </is>
       </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>A. There is a section or annex devoted to the situation analysis.
+B. The analysis cites sources (studies, official data, evaluations, consultations).
+C. The problem is bounded in scope, magnitude and affected population.</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ (T2 ∨ T3 ∨ T4)   but ¬ (T2 ∧ (T3 ∨ T4))</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   OR   T1 ∧ ¬T2 ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>"situation analysis"; "problem statement"; bibliographic citations; figures with %, USD or N=</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="320" customHeight="1" s="17">
       <c r="A10" s="2" t="inlineStr">
@@ -1756,6 +1942,28 @@
 T2: Are the causes supported by evidence or consultation (citation / reference)? (yes/no)
 T3: Is the project strategy explicitly mapped to causes (not only to symptoms)? (yes/no)
 DECISION: T1 ∧ T3</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>A. It distinguishes immediate, underlying and structural causes (or an equivalent scheme).
+B. The causes are linked to evidence or consultation.
+C. The project strategy relates to causes, not only to symptoms.</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T3   OR   ¬T1 ∧ T3</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>"immediate/underlying/structural causes"; "problem tree"; "root of the problem"</t>
         </is>
       </c>
     </row>
@@ -1886,6 +2094,29 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>A. Identifies the affected population group by name and magnitude.
+B. Gender analysis of the context (covering at least one of: roles, sexual division of labour, opportunities and constraints differentiated by sex).
+C. Sex-disaggregated data where available.</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬T3   (T2 is present but disaggregated data are missing)
+    OR    T1 ∧ T3 ∧ generic-T2 (T2 without specificity to the context)</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>"gender analysis"; "gender roles"; "sexual division of labour"; data broken down "women/men" or "F/M"</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="320" customHeight="1" s="17">
       <c r="A12" s="2" t="inlineStr">
@@ -2004,6 +2235,30 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ (T4 ∨ NA)</t>
         </is>
       </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>A. Stakeholder mapping (institutional, social, beneficiaries).
+B. Constraints and interests of each relevant actor.
+C. Explicit inclusion of women's organizations.
+D. Explicit inclusion of organizations of persons with disabilities where the project affects them.
+E. Analysis of power/influence among actors.</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬(T3 ∧ T4)</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   OR   ¬T2 (a list only, without analysis)</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>"stakeholder mapping"; "stakeholder analysis"; names of OPDs, women's organizations</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="320" customHeight="1" s="17">
       <c r="A13" s="2" t="inlineStr">
@@ -2130,6 +2385,35 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ (T4 ∨ NA)</t>
         </is>
       </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>A. Documented consultation plan with a methodology.
+B. Specific inclusion of marginalised groups (not merely a list).
+C. Measures for equitable participation (accessibility, translation, scheduling).
+D. Analysis of potential discriminatory effects and their mitigation.
+E. Free, prior and informed consent for indigenous peoples where applicable (FPIC).</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬T3   OR   T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   OR   consultation only with authorities/partners, without marginalised groups</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>E applies only if the project affects indigenous peoples — this must be documented.</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>"FPIC"; "free, prior and informed consent"; "interpretation"; "accessible language"; names of marginalised groups</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="320" customHeight="1" s="17">
       <c r="A14" s="2" t="inlineStr">
@@ -2244,6 +2528,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>A. Explicit reference to the ILO's normative identity (conventions, recommendations).
+B. Explicit reference to tripartism (constituents: government, employers, workers).
+C. A value-added argument specific to the project (not generic).</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∨ ¬T2</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>"normative", "tripartite", "employers and workers", "ILO constituents"; conventions cited by number</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="320" customHeight="1" s="17">
       <c r="A15" s="2" t="inlineStr">
@@ -2358,6 +2664,27 @@
 T1: Does it describe the ILO's presence in the country (office, team, length of presence)? (yes/no)
 T2: Does it list ≥2 past or ongoing projects with title or code? (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>A. Description of the ILO's presence in the country (office, team).
+B. List or summary of relevant past/ongoing projects.</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∨ T2 (only one is met)</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>"ILO Office in"; names of past projects; project codes</t>
         </is>
       </c>
     </row>
@@ -2482,6 +2809,28 @@
 T2: Does it link at least one lesson to a visible decision in the present design? (yes/no)
 T3 (optional): Does it draw out concrete lessons, as a list or in prose? (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>A. Cites specific evaluations (project, country programme, strategy).
+B. (Optional) Draws out concrete lessons learned.
+C. Links those lessons to design decisions in the present project.</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   (cites but does not link)</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   OR   only "lessons have been taken into account" without a citation</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>"evaluation of", "lessons learned"; years; ievaldiscovery URLs</t>
         </is>
       </c>
     </row>
@@ -2619,6 +2968,35 @@
 DECISION: (#true of T1/T2/T3) ≥ 2</t>
         </is>
       </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>A. Sub-objective, outcome or output whose title names disability.
+B. Indicator disaggregated by disability or measuring it specifically.
+C. Activity whose main purpose is disability.
+D. (Optional, depending on the nature of the project) Budget line for disability.
+E. (Optional, depending on the nature of the project) Quantifiable target relating to disability.</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>DECISION: (#true of T1/T2/T3) = 1   OR   only T4/T5 without T1/T2/T3</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>DECISION: (#true of T1/T2/T3/T4/T5) = 0</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>Document where the project explicitly justifies that disability does not apply.</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>"persons with disabilities"; "PwD"; "accessibility"; "disaggregated by disability"</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="320" customHeight="1" s="17">
       <c r="A18" s="2" t="inlineStr">
@@ -2741,6 +3119,30 @@
 DECISION: T1 ∧ T2 ∧ (T3 ∨ T4)</t>
         </is>
       </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>A. Cites conventions/recommendations by number (e.g. C111, C190).
+B. Those instruments are integrated into the strategy (not merely listed).
+C. Indicators or objectives link to those instruments.
+D. Actions promoting ratification/application/awareness.
+E. References to NORMLEX or other legal sources.</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   (cited in the background but not integrated into the strategy)</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   (does not cite conventions by number)</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>"C087", "C098", "C190"; "Convention No."; "NORMLEX"; normlex.ilo.org URL</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="320" customHeight="1" s="17">
       <c r="A19" s="2" t="inlineStr">
@@ -2867,6 +3269,33 @@
 T2: Does it cite conclusions of the Committee on the Application of Standards or the Committee on Freedom of Association? (yes/no)
 T3: Do the cited observations inform the justification or the strategy (explicit link)? (yes/no)
 DECISION: (T1 ∨ T2) ∧ T3</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>A. Cites CEACR observations/direct requests concerning the country.
+B. Cites conclusions of the Committee on the Application of Standards or the Committee on Freedom of Association where applicable.
+C. Those observations inform the project's justification or strategy (an explicit link, not decorative).</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>DECISION: (T1 ∨ T2) ∧ ¬T3   (cites observations without linking them to the strategy)</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Document where the project has no link to ILS.</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>"CEACR"; "Committee of Experts"; "Committee on Freedom of Association"; "Committee on the Application of Standards"</t>
         </is>
       </c>
     </row>
@@ -2998,6 +3427,35 @@
 DECISION: T1 ∧ (#true of T2/T3/T4) ≥ 2 ∧ (T5 ∨ NA)</t>
         </is>
       </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>A. Explicit commitment to ILS compliance within the project.
+B. Fair wages specified (legal or sectoral reference).
+C. OSH conditions applicable to project staff and contractors.
+D. Grievance mechanism accessible to workers.
+E. Compliance clauses in third-party contracts.</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ exactly 1 of T2/T3/T4   OR   T5 absent where third parties are engaged</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   OR   only a general statement with no operational elements</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>If the project engages no workers directly or indirectly, document why this does not apply.</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>"wages", "OSH", "occupational safety and health", "grievance mechanism", "code of conduct"</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="320" customHeight="1" s="17">
       <c r="A21" s="2" t="inlineStr">
@@ -3129,6 +3587,35 @@
 T4: Sustainable practices in implementation (materials / energy / waste)? (yes/no)
 T5 (cond): if there is infrastructure/construction → specific environmental safety measures? (yes/no/NA)
 DECISION: T1 ∧ T2 ∧ (#true of T3/T4) ≥ 1 ∧ (T5 ∨ NA)</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>A. Analysis of the project's potential environmental impacts.
+B. Measures to mitigate the impacts identified.
+C. Consideration of biodiversity and affected communities.
+D. Sustainable practices in implementation (materials, energy, waste).
+E. Where there is infrastructure/construction: specific environmental safety measures.</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   OR   T1 ∧ T2 ∧ ¬T5 (where T5 applies)</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   (decorative mentions only)</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>If the project is 100% normative/advisory with no physical activities, document it but still assess A.</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>"environmental impact"; "biodiversity"; "waste"; "energy"; "environmental sustainability"</t>
         </is>
       </c>
     </row>
@@ -3286,6 +3773,58 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>A. Distinguishes gender-sensitive / responsive / transformative approaches.
+B. Explicitly articulates how the project challenges gender norms or power relations.
+C. DEDICATED actions to transform relations (not merely to include women).
+D. Indicators measure changes in relations, not only numerical participation.
+E. Cites technical guidance (e.g. "Practical Guide" No. 15).</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>DECISION: (T1 ∨ T3) ∧ ¬(T1 ∧ T2 ∧ T3)
+FLOOR RULE (T3): if T3 is TRUE, the result can NEVER be "No".
+With T3 true, the result is "Yes" only if T1 and T2 are also met; in any
+other case the result is, at minimum, "Partial".
+Rationale: T3 evidences DEDICATED actions to transform gender relations.
+That substance prevails over nomenclature. A PRODOC that carries out
+dedicated transformative actions cannot be rated "No" for failing to label
+them with the sensitive/responsive/transformative taxonomy (T1 false), nor
+for failing to spell out the mechanism by which norms are challenged
+(T2 false).
+Cases this rule sends to "Partial":
+- T3 true and T1 false: dedicated actions exist, without distinguishing the approach.
+- T3 true and T2 false: dedicated actions exist, without articulating how they
+  challenge norms or power relations.
+- T1 true and ¬(T2 ∧ T3): the approach is declared but the actions remain
+  numerical or merely inclusive.</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ ¬T3
+"No" requires BOTH conditions to hold: the document does not distinguish the
+type of approach (T1 false) AND it presents no dedicated actions to transform
+gender relations (T3 false).
+If T3 is true, "No" is ruled out by the FLOOR RULE (see Partial), whatever the
+values of T1 and T2.
+Typical "No" case: the document only states that it "mainstreams gender", or
+uses generic equality formulations, with no dedicated actions and no
+distinction of approach.</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>If the context does not allow a transformative approach, this must be explicitly justified.</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>"transformative approach", "power relations", "gender norms", "Practical Guide No. 15"</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="320" customHeight="1" s="17">
       <c r="A23" s="5" t="inlineStr">
@@ -3407,6 +3946,29 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4</t>
         </is>
       </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>A. Describes the consultation/participation process during design (what, when, with whom).
+B. Lists the constituents consulted (government, employers, workers).
+C. Defines the parties' role in monitoring.
+D. Defines the parties' role in implementation.</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬(T3 ∧ T4)</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∨ ¬T2</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>names of ministries; trade union confederations; employers' chambers; "in monitoring", "in implementation"</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="320" customHeight="1" s="17">
       <c r="A24" s="5" t="inlineStr">
@@ -3524,6 +4086,29 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4 for ALL key stakeholders</t>
         </is>
       </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>A. Key stakeholders identified by name.
+B. Each stakeholder's link to the final beneficiaries.
+C. Role in relation to the problem (cause, affected, mitigator).
+D. Role in relation to the solution (implementer, validator, beneficiary).</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ (T2 ∨ T3 ∨ T4) but not all three for all stakeholders</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   (a list only, without analysis)</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>stakeholder table; columns "role", "interest", "link"</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="320" customHeight="1" s="17">
       <c r="A25" s="5" t="inlineStr">
@@ -3642,6 +4227,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>A. Explicit mention of consultation with ACT/EMP.
+B. Explicit mention of consultation with ACTRAV.
+C. The outcome of the consultation is integrated into the design.</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>DECISION: (T1 ∨ T2) ∧ ¬T3   OR   T1 ∧ T2 ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>"ACT/EMP"; "ACTRAV"; "specialists consulted"; specific names</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="320" customHeight="1" s="17">
       <c r="A26" s="5" t="inlineStr">
@@ -3760,6 +4367,28 @@
 T2: Does it list concrete commitments made by partners? (yes/no)
 T3 (optional): Are those commitments operational (time / resources / decisions)? (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>A. Describes the consultations held (when, with whom, on what).
+B. Lists concrete commitments made by partners.
+C. (Optional) Those commitments are operational (time, resources, decisions) — not merely declaratory.</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   OR   only claims of ownership without commitments</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>"minutes of meeting", "MoU", "letter of intent"; consultation dates</t>
         </is>
       </c>
     </row>
@@ -3887,6 +4516,28 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4</t>
         </is>
       </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>A. Evidence of acceptance of the objectives by each key partner.
+B. Acceptance of the performance framework / indicators.
+C. Acceptance of obligations and responsibilities.</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>DECISION: (T1 ∨ T2 ∨ T3) ∧ ¬T4   (asserted without documentary support)</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ ¬T2 ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>"MoU", "letter of intent", "cooperation agreement"; references to annexes</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="320" customHeight="1" s="17">
       <c r="A28" s="5" t="inlineStr">
@@ -4003,6 +4654,28 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4</t>
         </is>
       </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>A. Explicit strategy for continuous ownership (not merely one-off events).
+B. Shared governance mechanisms (committees, steering groups).
+C. Link to the sustainability strategy.</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ (T3 ∨ T4) but not both</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>"steering committee", "coordination group"</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="320" customHeight="1" s="17">
       <c r="A29" s="5" t="inlineStr">
@@ -4117,6 +4790,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>A. Capacity assessment carried out OR planned, with a methodology.
+B. Explicit conclusions (existing capacities vs gaps).
+C. Those conclusions inform the project design.</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   OR   only a vague statement, "capacities will be assessed"</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>"capacity assessment", "gap analysis"</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="320" customHeight="1" s="17">
       <c r="A30" s="5" t="inlineStr">
@@ -4235,6 +4930,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>A. Individual (technical) capacities.
+B. Organizational capacities (systems, processes).
+C. Enabling environment (legal framework, policies, financing).</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>DECISION: 2 of T1/T2/T3   OR   all 3 but with an almost exclusive emphasis on T1 (individual training)</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>DECISION: T1 only   (reduces capacity development to workshops)</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>"individual / organizational capacities / enabling environment"; "systemic"; "policy"</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="320" customHeight="1" s="17">
       <c r="A31" s="5" t="inlineStr">
@@ -4353,6 +5070,27 @@
 T1: Explicit evidence of constituents' interest in the post-project period? (yes/no)
 T2: Is that evidence concrete (letter, MoU, allocation of future staff/budget)? (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>A. Evidence of explicit constituent interest in the post-project period.
+B. That evidence is concrete (letter, MoU, allocation of future staff/budget).</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   (a statement without operationalisation)</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>"post-project", "sustainability", letters of commitment, future budget allocations</t>
         </is>
       </c>
     </row>
@@ -4479,6 +5217,29 @@
 DECISION: T1   (an explicit plan suffices; T2–T5 raise the score)</t>
         </is>
       </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>A. Institutional mechanism (training of trainers, integration into existing systems).
+B. Financial mechanism (post-project funding sources).
+C. Governance mechanism (who sustains the results).
+D. Transition timetable.</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ any of T2/T3/T4/T5   (scattered elements without an integrated plan)</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ no operational element</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>"sustainability plan"; "sustaining results"</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="320" customHeight="1" s="17">
       <c r="A33" s="5" t="inlineStr">
@@ -4607,6 +5368,34 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4 ∧ T5</t>
         </is>
       </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>A. The proposal identifies the preconditions for scaling up.
+B. Defines objective success criteria.
+C. Plan for measuring/demonstrating success.
+D. Plan for transition to the scale-up phase.</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ T3 ∧ ¬(T4 ∧ T5)</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2 ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 (no test phase is defined) → explicit N/A</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>"pilot", "test phase", "proof of concept", "scale-up"</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="320" customHeight="1" s="17">
       <c r="A34" s="5" t="inlineStr">
@@ -4719,6 +5508,28 @@
 T2: An identified source of financial resources after the project? (yes/no)
 T3: A plausibility argument with support (existing sectoral budget, institutional commitment)? (yes/no)
 DECISION: T1 ∧ T2 ∧ T3</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>A. Identifies the source of human resources after the project.
+B. Identifies the source of financial resources after the project.
+C. Argues plausibility (not merely declaratory).</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>DECISION: (T1 ∨ T2) ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>"post-project resources", "sectoral budget", "budget line"</t>
         </is>
       </c>
     </row>
@@ -4847,6 +5658,29 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4</t>
         </is>
       </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>A. Explicit exit strategy.
+B. Plan for transferring responsibilities (what, to whom, when).
+C. Capacity development actions specific to the transfer.
+D. Exit timetable.</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬(T3 ∧ T4)</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>"exit strategy", "transfer of responsibilities"</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="320" customHeight="1" s="17">
       <c r="A36" s="8" t="inlineStr">
@@ -4968,6 +5802,29 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4</t>
         </is>
       </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>A. The outputs → outcomes → impact causal chain is made explicit.
+B. Mechanisms of change identified (not merely arrows).
+C. Critical assumptions stated.
+D. Discursive emphasis on results (not on a list of activities).</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ T3 ∧ ¬T4   (a clear chain but the focus is on activities)</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   (the logic can only be inferred from the activity list)</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>"theory of change", "ToC", "mechanism of change", "critical assumption", "if X then Y"</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="320" customHeight="1" s="17">
       <c r="A37" s="8" t="inlineStr">
@@ -5091,6 +5948,28 @@
 DECISION: T1 ∨ T2 ∨ T3   (at least one; subjectivity acknowledged)</t>
         </is>
       </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>A. Coverage: the outputs cover the outcomes with no logical gaps.
+B. Sufficiency: each outcome has outputs that justify achieving it.
+C. The outcomes → impact link is reasoned.</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>DECISION: partial traceability exists but there are gaps in ≥1 outcome</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>DECISION: pervasive gaps; outputs and outcomes are decoupled</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>"logical framework", "logframe"; verbs connecting rows</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="320" customHeight="1" s="17">
       <c r="A38" s="8" t="inlineStr">
@@ -5205,6 +6084,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>A. Specific actors of capacity development are named.
+B. Type of change expected (performance, behaviour, practices).
+C. Mechanism by which capacity translates into change.</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>DECISION: only "capacities will be developed", without specifying</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>"behavioural change", "improved performance", "practical application"</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="320" customHeight="1" s="17">
       <c r="A39" s="8" t="inlineStr">
@@ -5323,6 +6224,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>A. Assumptions stated explicitly.
+B. Assumptions tied to levels of the chain (outputs / outcomes / impact).
+C. Reference to past or parallel interventions (ILO or other actors).</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   (generic assumptions)</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   OR   assumptions confused with risks</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>"assumption", "it is assumed", "precondition"</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="320" customHeight="1" s="17">
       <c r="A40" s="8" t="inlineStr">
@@ -5441,6 +6364,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>A. Cites specific evaluations (project, programme, study).
+B. Those evaluations support causal links in the logical framework.
+C. The lessons are explicitly applied to the present design.</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬(T2 ∧ T3)</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>"evaluation", "meta-evaluation", "ievaldiscovery", evaluation years</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="320" customHeight="1" s="17">
       <c r="A41" s="8" t="inlineStr">
@@ -5554,6 +6499,27 @@
 T1: Do the outcomes express states / situations ("X is strengthened", "Y has access")? (yes/no)
 T2: Absence of activity formulations ("through", "by means of", "by carrying out") in &gt;80% of the outcomes. (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>A. Outcome statements express states/situations (X is strengthened, Y has access).
+B. Absence of activity formulations ("through", "by means of", "by carrying out").</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   (a mix of change and action language)</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   (action language predominates)</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>"is strengthened", "has access", "has been improved"; absence of "through", "by means of"</t>
         </is>
       </c>
     </row>
@@ -5676,6 +6642,30 @@
 DECISION: ALL outcomes meet S+M+A+R+T</t>
         </is>
       </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>S — Specific (what exactly).
+M — Measurable (with what indicator and threshold).
+A — Achievable (feasible with the resources).
+R — Relevant (linked to the problem and the ToC).
+T — Time-bound (with a defined deadline).</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>DECISION: outcomes meet 3–4 SMART attributes; typically M or T is missing</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>DECISION: outcomes are aspirations (≤2 attributes)</t>
+        </is>
+      </c>
+      <c r="AB42" t="inlineStr">
+        <is>
+          <t>indicators with a figure/%, deadlines "by 2026", "by the end of the project"</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="320" customHeight="1" s="17">
       <c r="A43" s="8" t="inlineStr">
@@ -5785,6 +6775,27 @@
 T1: Are outputs framed as deliverables ("Document X published", "N people certified")? (yes/no)
 T2: Absence of activity formulations ("Hold workshops", "Train…") in &gt;80% of the outputs. (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>A. Outputs framed as deliverables ("Document X published", "N people certified").
+B. Absence of activity formulations ("Hold workshops", "Train…").</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   (mixes outputs and activities)</t>
+        </is>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>"published", "certified", "delivered"; absence of "carry out", "undertake"</t>
         </is>
       </c>
     </row>
@@ -5920,6 +6931,33 @@
   if T4=no  → T2 ∨ T3</t>
         </is>
       </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>A. Outcome or output whose title names gender/equality/women.
+B. Indicator disaggregated by sex or gender-specific.
+C. Quantifiable target by sex or on gender.</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>DECISION: appears only in assumptions or in the framework's cross-cutting language; no DEDICATED element</t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>DECISION: the logical framework mentions gender neither in outcomes, outputs nor indicators</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>Only if the CPO gender marker is 0 — this must be documented.</t>
+        </is>
+      </c>
+      <c r="AB44" t="inlineStr">
+        <is>
+          <t>"gender equality", "sex-disaggregated", "GEM"; outcome titles naming gender</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="320" customHeight="1" s="17">
       <c r="A45" s="8" t="inlineStr">
@@ -6053,6 +7091,33 @@
   if T4=no  → T2 ∨ T3</t>
         </is>
       </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>A. Outcome or output that names disability.
+B. Disability-specific or disaggregated indicator.
+C. Quantifiable disability target.</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>DECISION: mentioned only at the level of assumptions or cross-cutting language; no DEDICATED element</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>DECISION: the logical framework does not include disability</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>Only if the CPO disability label does not apply — this must be documented.</t>
+        </is>
+      </c>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>"disability inclusion", "disaggregated by disability", "PwD"</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="320" customHeight="1" s="17">
       <c r="A46" s="8" t="inlineStr">
@@ -6166,6 +7231,27 @@
 T1: Is there a risk analysis section or annex? (yes/no)
 T2: Are the risks categorised (strategic / operational / fiduciary / contextual / reputational)? (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>A. There is a risk analysis section or annex.
+B. The risks are categorised (strategic, operational, fiduciary, contextual).</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB46" t="inlineStr">
+        <is>
+          <t>"risk matrix", "risk analysis", categories ("operational", "fiduciary")</t>
         </is>
       </c>
     </row>
@@ -6292,6 +7378,30 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4 ∧ (T5 ∨ NA)</t>
         </is>
       </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>A. SEA-specific risks identified.
+B. Prevention mechanisms (codes of conduct, mandatory training).
+C. Accessible and confidential reporting mechanism.
+D. Response protocol and victim support.
+E. SEA clauses in third-party contracts.</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬(T3 ∧ T4)</t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>DECISION: states only "zero tolerance", without operationalisation</t>
+        </is>
+      </c>
+      <c r="AB47" t="inlineStr">
+        <is>
+          <t>"SEA", "sexual exploitation and abuse", "PSEA", "code of conduct", "reporting mechanism"</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="320" customHeight="1" s="17">
       <c r="A48" s="8" t="inlineStr">
@@ -6418,6 +7528,35 @@
 DECISION: T1 ∧ T2 ∧ T4 ∧ (T3 ∨ NA)</t>
         </is>
       </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>A. Identification of community risks (not only risks to project staff; not cross-cutting).
+B. Measures for physical and environmental risks (traffic, hazardous materials, pollution; cross-cutting component: Environment).
+C. Where there is security personnel: use-of-force and abuse-prevention protocol (conditional; not cross-cutting).
+D. Community grievance mechanism (not cross-cutting).
+Note: apply DEDICATED vs FRAMING only to the environmental evidence. Do not treat community risks, OSH or security as cross-cutting themes.</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>DECISION: covers only risks to staff, not to the community; or T1∧T2 ∧ ¬T4</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>If the project is 100% remote/normative with no physical presence, document it.</t>
+        </is>
+      </c>
+      <c r="AB48" t="inlineStr">
+        <is>
+          <t>"community health and safety", "community risks", "pollution", "hazardous materials", "community grievance mechanism"</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="320" customHeight="1" s="17">
       <c r="A49" s="8" t="inlineStr">
@@ -6537,6 +7676,28 @@
 DECISION: T1 ∧ T3   (T2 raises the score but is not required)</t>
         </is>
       </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>A. Identifies ILS non-compliance risks in the project context.
+B. Links to CEACR observations or other supervisory bodies.
+C. Specific mitigation plan.</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB49" t="inlineStr">
+        <is>
+          <t>"non-compliance", "compliance risks", "CEACR", conventions by number</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="320" customHeight="1" s="17">
       <c r="A50" s="8" t="inlineStr">
@@ -6659,6 +7820,32 @@
 T1: Is the project budget &gt; USD 1,000,000? (yes/no/NA)
 T2: Is a risk register in the current ILO format attached? (yes/no)
 DECISION: if T1=yes → T2; if T1=no → N/A</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>A. Risk register in the current ILO format.
+B. Attached to the proposal (as an annex, not merely referenced).</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ a register is present but not the current version, or not attached though referenced</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 (budget ≤ USD 1M)</t>
+        </is>
+      </c>
+      <c r="AB50" t="inlineStr">
+        <is>
+          <t>"risk register", total budget in USD</t>
         </is>
       </c>
     </row>
@@ -6777,6 +7964,28 @@
 T2: Are likelihood and impact rated (numerical or categorical scale)? (yes/no)
 T3: Are the risks material to the project's success? (yes/no)
 DECISION: T1 ∧ T2 ∧ T3</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>A. Specificity: each risk is contextual to the project, not a generic template.
+B. Likelihood and impact rated.
+C. Risks material to the project's success.</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>DECISION: some risks specific, others generic; or the rating is missing</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>DECISION: the risks are institutional boilerplate, without contextualisation</t>
+        </is>
+      </c>
+      <c r="AB51" t="inlineStr">
+        <is>
+          <t>"high/medium/low likelihood", "impact", "1–5 scale"</t>
         </is>
       </c>
     </row>
@@ -6893,6 +8102,28 @@
 DECISION: T1 ∧ T2 ∧ T3 for ALL medium/high risks</t>
         </is>
       </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>A. Each medium/high risk has a mitigation measure.
+B. Each measure has an owner.
+C. Each measure has a monitoring method.</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>DECISION: T1 universal but T2 or T3 missing for several risks</t>
+        </is>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>DECISION: medium/high risks with no measures, or only generic measures</t>
+        </is>
+      </c>
+      <c r="AB52" t="inlineStr">
+        <is>
+          <t>columns "measure", "owner", "monitoring" in the risk matrix</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="320" customHeight="1" s="17">
       <c r="A53" s="8" t="inlineStr">
@@ -7020,6 +8251,34 @@
 DECISION: T1 ∧ T2 ∧ (T3 ∨ NA)</t>
         </is>
       </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>A. Collection system described (what data, how often, by whom).
+B. Justification of the resources allocated to M&amp;E.
+C. Evaluability review where applicable (project above the threshold).
+D. (Optional) Project learning plan.</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>DECISION: "monitoring will be carried out", with no system described</t>
+        </is>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>Document the threshold criterion for C.</t>
+        </is>
+      </c>
+      <c r="AB53" t="inlineStr">
+        <is>
+          <t>"M&amp;E system", "evaluability", "learning plan", "MEL"</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="320" customHeight="1" s="17">
       <c r="A54" s="8" t="inlineStr">
@@ -7137,6 +8396,29 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4</t>
         </is>
       </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>A. Feedback loop defined (data → decisions).
+B. Information needs for reporting specified.
+C. Responsible staff named or identified by post.
+D. Frequency of the review cycles.</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T3 ∧ ¬(T2 ∧ T4)</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   (data are collected with no defined use)</t>
+        </is>
+      </c>
+      <c r="AB54" t="inlineStr">
+        <is>
+          <t>"feedback loop", "quarterly review", "half-yearly report"</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="320" customHeight="1" s="17">
       <c r="A55" s="8" t="inlineStr">
@@ -7252,6 +8534,29 @@
 T3: Are analysis methods specified? (yes/no)
 T4: Roles and responsibilities per method/indicator? (yes/no)
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>A. M&amp;E plan as a discrete document or section.
+B. Collection methods named (survey, interview, administrative records).
+C. Analysis methods specified.
+D. Roles and responsibilities per method/indicator.</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬(T3 ∧ T4)</t>
+        </is>
+      </c>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   OR   only an indicator table, without methods</t>
+        </is>
+      </c>
+      <c r="AB55" t="inlineStr">
+        <is>
+          <t>"collection method", "qualitative/quantitative analysis", "roles"</t>
         </is>
       </c>
     </row>
@@ -7388,6 +8693,31 @@
 DECISION: ALL indicators satisfy T1+T2+T3+T4+T5+T6</t>
         </is>
       </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>A. SMART indicators (all five attributes).
+B. Gender-sensitive (sex-disaggregated or gender-specific).
+C. Allow for disability inclusion (disaggregated or specific).
+D. Baseline for each indicator.
+E. Target and milestones defined.
+F. Coverage of the outcomes (not only outputs).</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T4 ∧ T5 ∧ T6 but T2/T3 are generic (inclusive in language without real disaggregation)</t>
+        </is>
+      </c>
+      <c r="Z56" t="inlineStr">
+        <is>
+          <t>DECISION: indicators are not SMART, lack a baseline, or ignore gender/disability</t>
+        </is>
+      </c>
+      <c r="AB56" t="inlineStr">
+        <is>
+          <t>"SMART", "disaggregated by sex / disability", "baseline", "target", "milestone"</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="320" customHeight="1" s="17">
       <c r="A57" s="8" t="inlineStr">
@@ -7508,6 +8838,27 @@
 T1: Is the evaluation budget line SEPARATE and named? (yes/no)
 T2: Is the amount ≥ ~2% of the total budget (or is a departure justified)? (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>A. Separate evaluation budget line.
+B. Amount ≥ ~2% of the total budget (or a justification if it differs).</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   OR   an identifiable amount without a separate budget line</t>
+        </is>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   (no budget line and no identifiable amount)</t>
+        </is>
+      </c>
+      <c r="AB57" t="inlineStr">
+        <is>
+          <t>"evaluation budget", "evaluation line", percentage of the total</t>
         </is>
       </c>
     </row>
@@ -7638,6 +8989,33 @@
 DECISION: T2 ∧ T3 ∧ (T1 ∨ NA)</t>
         </is>
       </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>A. Where there is an inception phase: activities and results of the initial period made explicit.
+B. Overall timeframe justified against complexity and capacities.
+C. Timetable with quarterly or half-yearly milestones.</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>DECISION: T3 ∧ ¬T2   (a timetable without justification)</t>
+        </is>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T3</t>
+        </is>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>Document where there is no inception phase.</t>
+        </is>
+      </c>
+      <c r="AB58" t="inlineStr">
+        <is>
+          <t>"inception", "initial phase", "timetable", "Gantt", "quarterly milestones"</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="320" customHeight="1" s="17">
       <c r="A59" s="8" t="inlineStr">
@@ -7756,6 +9134,28 @@
 T2: Is there consistency between logical framework activities and budget lines? (yes/no)
 T3 (optional): Are unit costs or calculations visible? (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>A. Budget broken down by activity or output.
+B. Consistency between logical framework activities and budget lines.
+C. (Optional) Unit costs or calculations visible.</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>DECISION: budget only at the level of broad categories</t>
+        </is>
+      </c>
+      <c r="AB59" t="inlineStr">
+        <is>
+          <t>"breakdown by activity", "BoQ", "cost driver", "unit cost"</t>
         </is>
       </c>
     </row>
@@ -7879,6 +9279,34 @@
 DECISION: ALL applicable items (T1–T4) have a specific budget line with an amount</t>
         </is>
       </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>A. Budget line for a gender specialist where applicable.
+B. Budget line for a disability specialist where applicable.
+C. Budget line for information accessibility (plain language, alternative formats).
+D. Budget line for interpretation into local languages or sign language where applicable.</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>DECISION: the need is acknowledged but left as "if required", with no budget line</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>DECISION: no budget lines and no recognition of cross-cutting costs</t>
+        </is>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>Document item by item where it does not apply.</t>
+        </is>
+      </c>
+      <c r="AB60" t="inlineStr">
+        <is>
+          <t>"gender/disability specialist", "accessibility", "local language", "sign language"</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="320" customHeight="1" s="17">
       <c r="A61" s="8" t="inlineStr">
@@ -7988,6 +9416,27 @@
 T1: An explicit mention of cost-effectiveness or "value for money"? (yes/no)
 T2: Is it linked to the project design (not only to administration)? (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>A. Explicit mention of cost-effectiveness or "value for money".
+B. Linked to the design (not only to administration).</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="Z61" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB61" t="inlineStr">
+        <is>
+          <t>"cost-effectiveness", "value for money", "efficiency"</t>
         </is>
       </c>
     </row>
@@ -8108,6 +9557,28 @@
 DECISION: T1 ∧ T2 ∧ (T3 ∨ NA)</t>
         </is>
       </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>A. Analysis of design alternatives with costs/benefits.
+B. Justification of the option chosen.
+C. Where applicable: comparison against benchmarks (similar projects).</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>DECISION: T2 ∧ ¬T1   (justifies without comparing alternatives)</t>
+        </is>
+      </c>
+      <c r="Z62" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="AB62" t="inlineStr">
+        <is>
+          <t>"analysis of alternatives", "benchmark", "cost-benefit"</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="320" customHeight="1" s="17">
       <c r="A63" s="11" t="inlineStr">
@@ -8222,6 +9693,28 @@
 DECISION: T1 ∧ (T2 ∨ T3)</t>
         </is>
       </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>A. Identifies the managing office/unit.
+B. Where management is regional/national: a field office close to the beneficiaries.
+C. Where management is centralised: explicit justification on effectiveness grounds.</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T3 (centralisation without justification)</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB63" t="inlineStr">
+        <is>
+          <t>"field office", "headquarters", "decentralised", "justification for centralisation"</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="320" customHeight="1" s="17">
       <c r="A64" s="11" t="inlineStr">
@@ -8336,6 +9829,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>A. Organigram or description of staff roles.
+B. Explicit line of accountability (who reports to whom).
+C. Responsible ILO official identified by post or name.</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬(T2 ∧ T3)</t>
+        </is>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>DECISION: only "staff will be recruited as required"</t>
+        </is>
+      </c>
+      <c r="AB64" t="inlineStr">
+        <is>
+          <t>"organigram", "reports to", "responsible ILO official", specific names/posts</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="320" customHeight="1" s="17">
       <c r="A65" s="11" t="inlineStr">
@@ -8454,6 +9969,27 @@
 T1: Does it identify the technical or administrative units that will provide support? (yes/no)
 T2: Is that support budgeted for (a line or allocation)? (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>A. Identifies the technical or administrative units that will provide support.
+B. That support is budgeted for (a line or allocation).</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>DECISION: assumes support without provision or identification</t>
+        </is>
+      </c>
+      <c r="AB65" t="inlineStr">
+        <is>
+          <t>"backstopping", "technical unit", "administrative support", unit names (PROGRAM, ENTERPRISES, …)</t>
         </is>
       </c>
     </row>
@@ -8580,6 +10116,29 @@
 T3: Financial and reporting systems? (yes/no)
 T4: Levels of authority and approval? (yes/no)
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>A. Staffing plan.
+B. Procurement procedures (ILO standards or adaptations).
+C. Financial and reporting systems.
+D. Levels of authority and approval.</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>DECISION: 2–3 of T1/T2/T3/T4</t>
+        </is>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>DECISION: only "ILO procedures will apply"</t>
+        </is>
+      </c>
+      <c r="AB66" t="inlineStr">
+        <is>
+          <t>"procurement", "IRIS", "levels of authority"</t>
         </is>
       </c>
     </row>
@@ -8712,6 +10271,34 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4</t>
         </is>
       </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>A. Decent work clauses in third-party contracts.
+B. Fair employment clauses (wages, working time, freedom of association).
+C. Grievance mechanism accessible to third-party workers.
+D. Compliance monitoring by the ILO.</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬(T3 ∧ T4)</t>
+        </is>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>DECISION: only "third parties will comply with the standards"</t>
+        </is>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>DECISION: there are no contractors — document</t>
+        </is>
+      </c>
+      <c r="AB67" t="inlineStr">
+        <is>
+          <t>"contractor", "subcontractor", "decent work clause", "grievance mechanism"</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="320" customHeight="1" s="17">
       <c r="A68" s="11" t="inlineStr">
@@ -8826,6 +10413,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>A. Roles of each institution/partner made explicit.
+B. Implementation procedures (how they work together).
+C. Justification for the choice of partners (why these and not others).</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬T3</t>
+        </is>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>DECISION: lists partners only, without roles or justification</t>
+        </is>
+      </c>
+      <c r="AB68" t="inlineStr">
+        <is>
+          <t>"selection of partners", "selection criteria", "modus operandi"</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="320" customHeight="1" s="17">
       <c r="A69" s="11" t="inlineStr">
@@ -8941,6 +10550,27 @@
 DECISION: T1 ∧ T2</t>
         </is>
       </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>A. Explicit evidence of acceptance by each partner.
+B. Supporting document (letter, MoU, minutes).</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB69" t="inlineStr">
+        <is>
+          <t>"letter of acceptance", "signed MoU", "agreed minutes"</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="320" customHeight="1" s="17">
       <c r="A70" s="11" t="inlineStr">
@@ -9050,6 +10680,27 @@
 T1: An organizational capacity assessment carried out or planned, with a methodology? (yes/no)
 T2: An explicit reference in the proposal (not only in an uncited annex)? (yes/no)
 DECISION: T1 ∧ T2</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>A. Organizational capacity assessment carried out or planned.
+B. Explicit reference in the proposal (not only in an uncited annex).</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   (mentioned without method or findings)</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1</t>
+        </is>
+      </c>
+      <c r="AB70" t="inlineStr">
+        <is>
+          <t>"organizational capacity assessment", "OCA", "institutional assessment"</t>
         </is>
       </c>
     </row>
@@ -9170,6 +10821,33 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>A. Capacity development plan for the implementing partners.
+B. Operational components (training, mentoring, accompaniment).
+C. Gender-responsiveness component.</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬T3   (gender remains at framing level)</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>DECISION: gaps identified but no plan</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>DECISION: the assessment identified no gaps — document</t>
+        </is>
+      </c>
+      <c r="AB71" t="inlineStr">
+        <is>
+          <t>"institutional strengthening plan", "capacity development plan", "gender-responsive"</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="320" customHeight="1" s="17">
       <c r="A72" s="11" t="inlineStr">
@@ -9286,6 +10964,28 @@
 T2: A plausibility argument with evidence (not simply "they are competent")? (yes/no)
 T3 (cond): if demonstrated capacity is limited → specific mitigation? (yes/no/NA)
 DECISION: T1 ∧ T2 ∧ (T3 ∨ NA)</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>A. Partners' track record (similar projects, demonstrated capacity).
+B. Plausibility argument (not merely "they are competent").
+C. Mitigation where demonstrated capacity is limited.</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ ¬T2   OR   track record absent but the partners are well established</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>DECISION: merely asserts that they will deliver well</t>
+        </is>
+      </c>
+      <c r="AB72" t="inlineStr">
+        <is>
+          <t>"track record", "previous projects", "demonstrated capacity"</t>
         </is>
       </c>
     </row>
@@ -9405,6 +11105,29 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ T4</t>
         </is>
       </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>A. Stakeholder communication plan (what, when, how).
+B. Expected communication products (reports, briefings, events).
+C. Human resources allocated.
+D. Financial resources allocated.</t>
+        </is>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬(T3 ∧ T4)</t>
+        </is>
+      </c>
+      <c r="Z73" t="inlineStr">
+        <is>
+          <t>DECISION: "stakeholders will be informed", without operationalisation</t>
+        </is>
+      </c>
+      <c r="AB73" t="inlineStr">
+        <is>
+          <t>"communication plan", "briefing", "quarterly report"</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="320" customHeight="1" s="17">
       <c r="A74" s="11" t="inlineStr">
@@ -9517,6 +11240,28 @@
 T2 (alt): A development timetable, where the strategy is not yet drafted? (yes/no)
 T3: Expected products (press notes, social media, multimedia)? (yes/no)
 DECISION: (T1 ∧ T3)   OR   T2 with a clear timetable</t>
+        </is>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>A. Public communication strategy (not only a technical one).
+B. Development timetable where the strategy is not yet drafted.
+C. Expected products (press notes, social media, multimedia).</t>
+        </is>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>DECISION: announces a strategy without a timetable or products</t>
+        </is>
+      </c>
+      <c r="Z74" t="inlineStr">
+        <is>
+          <t>DECISION: no public communication strategy is included</t>
+        </is>
+      </c>
+      <c r="AB74" t="inlineStr">
+        <is>
+          <t>"communication strategy", "general public", "human interest"</t>
         </is>
       </c>
     </row>
@@ -9636,6 +11381,29 @@
 DECISION: T1 ∧ T2 ∧ T3 ∧ (T4 ∨ NA)</t>
         </is>
       </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>A. Human resources allocated to communication.
+B. Financial resources allocated.
+C. Formats accessible to persons with disabilities.
+D. Products in local languages / plain language / sign language where applicable.</t>
+        </is>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬T3   (accessibility declared without a budget line)</t>
+        </is>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1 ∧ ¬T2</t>
+        </is>
+      </c>
+      <c r="AB75" t="inlineStr">
+        <is>
+          <t>"accessibility", "alternative formats", "sign language", "local language"</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="320" customHeight="1" s="17">
       <c r="A76" s="11" t="inlineStr">
@@ -9759,6 +11527,32 @@
 DECISION: if T1 ∧ T2 → T3 ∧ T4; if ¬(T1 ∧ T2) → N/A</t>
         </is>
       </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>A. DCOMM template completed.
+B. Coordination with the relevant country office.</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ T3 ∧ ¬T4</t>
+        </is>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>DECISION: T1 ∧ T2 ∧ ¬T3 ∧ ¬T4</t>
+        </is>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>DECISION: ¬T1   OR   ¬T2</t>
+        </is>
+      </c>
+      <c r="AB76" t="inlineStr">
+        <is>
+          <t>"PPP", "public-private partnership", "European Commission", "DCOMM", budget in USD</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="320" customHeight="1" s="17">
       <c r="A77" s="14" t="inlineStr">
@@ -9873,6 +11667,28 @@
 DECISION: T1 ∧ T2 ∧ T3</t>
         </is>
       </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>A. All sections of the ILO template present.
+B. Order consistent with the guidance.
+C. Required annexes included.</t>
+        </is>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>DECISION: 2 of T1/T2/T3</t>
+        </is>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>DECISION: key sections or annexes are missing</t>
+        </is>
+      </c>
+      <c r="AB77" t="inlineStr">
+        <is>
+          <t>"Executive summary", "Background", "Logical framework", "Budget", "Annexes" — compare against the ILO template</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="320" customHeight="1" s="17">
       <c r="A78" s="14" t="inlineStr">
@@ -9989,6 +11805,28 @@
 T2: Absence of unnecessary jargon or evident repetition? (yes/no)
 T3: Visible structure (subheadings, tables, bullets where they help)? (yes/no)
 DECISION: T1 ∧ T2 ∧ T3</t>
+        </is>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>A. Core ideas identifiable without re-reading.
+B. Absence of unnecessary jargon or repetition.
+C. Visible structure (subheadings, tables, bullets where they help).</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>DECISION: mostly clear text but with dense or repetitive sections</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>DECISION: core ideas are buried; hard to follow</t>
+        </is>
+      </c>
+      <c r="AB78" t="inlineStr">
+        <is>
+          <t>executive summary, subheadings, paragraph length, tables vs prose</t>
         </is>
       </c>
     </row>

</xml_diff>